<commit_message>
Sync customer workbook to twelve entries
</commit_message>
<xml_diff>
--- a/dist/고객관리_연락처기준.xlsx
+++ b/dist/고객관리_연락처기준.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="Rb2e337d4849543f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R4d889e5a72e543b0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -964,7 +964,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="발굴일"/>
     <x:tableColumn id="2" name="고객명"/>
@@ -1224,7 +1224,7 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="14.399999618530273">
-      <x:c r="A5" s="5">
+      <x:c r="A5" s="7">
         <x:v>46306.5354914583</x:v>
       </x:c>
       <x:c r="B5" t="s">
@@ -1250,7 +1250,7 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="14.399999618530273">
-      <x:c r="A6" s="5">
+      <x:c r="A6" s="7">
         <x:v>46306.5354914583</x:v>
       </x:c>
       <x:c r="B6" t="s">
@@ -1377,6 +1377,140 @@
       </x:c>
       <x:c r="H10" t="str">
         <x:v>https://www.urt.co.kr/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="7" t="d">
+        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>뉴골드</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>통일상가</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>남성 캐주얼 바지</x:v>
+      </x:c>
+      <x:c r="E11" t="str"/>
+      <x:c r="F11" t="str"/>
+      <x:c r="G11" t="str">
+        <x:v>남성 캐주얼 바지 도매</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>공개 채용 공고 확인 · 연락처 확인 필요</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="7" t="d">
+        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>하프인치</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>디오트</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>여성 바지·원단</x:v>
+      </x:c>
+      <x:c r="E12" t="str"/>
+      <x:c r="F12" t="str"/>
+      <x:c r="G12" t="str">
+        <x:v>여성 팬츠·원단·패턴</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>공개 채용 공고 확인 · 연락처 확인 필요</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="7" t="d">
+        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>더베스트오버초이스</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>통일상가 B동 2층 250·251</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>가을·겨울 바지</x:v>
+      </x:c>
+      <x:c r="E13" t="str"/>
+      <x:c r="F13" t="str"/>
+      <x:c r="G13" t="str">
+        <x:v>가을·겨울 바지·재킷</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>고객관리 후보 기록 · 연락처 확인 필요</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="7" t="d">
+        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>디오트 여성 팬츠 매장 후보</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>디오트</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>여성복·바지</x:v>
+      </x:c>
+      <x:c r="E14" t="str"/>
+      <x:c r="F14" t="str">
+        <x:v>02-2117-8000</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>여성복·잡화 도매 상가</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>https://dongdaemunmarket.net/board/b03/47537</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="7" t="d">
+        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>누죤 여성 캐주얼 매장 후보</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>누죤</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>여성 캐주얼·바지</x:v>
+      </x:c>
+      <x:c r="E15" t="str"/>
+      <x:c r="F15" t="str"/>
+      <x:c r="G15" t="str">
+        <x:v>여성 캐주얼 의류 도매</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>동대문 도매시장 후보 · 업체별 연락처 확인 필요</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="7" t="d">
+        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>청평화상가 바지 매장 후보</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>청평화상가</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>바지·재킷</x:v>
+      </x:c>
+      <x:c r="E16" t="str"/>
+      <x:c r="F16" t="str"/>
+      <x:c r="G16" t="str">
+        <x:v>여성 의류·바지 도매</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>동대문 도매시장 후보 · 업체별 연락처 확인 필요</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1386,7 +1520,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd72f3dbefcd9477d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d5d91d18f5b4d02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Format discovery dates as date only
</commit_message>
<xml_diff>
--- a/dist/고객관리_연락처기준.xlsx
+++ b/dist/고객관리_연락처기준.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R4d889e5a72e543b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="Rea374cf68841420a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -86,13 +86,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <x:numFmt numFmtId="42" formatCode="_-&quot;₩&quot;* #,##0_-;\-&quot;₩&quot;* #,##0_-;_-&quot;₩&quot;* &quot;-&quot;_-;_-@_-"/>
     <x:numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <x:numFmt numFmtId="44" formatCode="_-&quot;₩&quot;* #,##0.00_-;\-&quot;₩&quot;* #,##0.00_-;_-&quot;₩&quot;* &quot;-&quot;??_-;_-@_-"/>
     <x:numFmt numFmtId="176" formatCode="yyyy/mm/dd\ h:mm:ss"/>
     <x:numFmt numFmtId="200" formatCode="yyyy/mm/dd"/>
+    <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
   <x:fonts count="26">
     <x:font>
@@ -710,7 +711,7 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="8">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
@@ -727,6 +728,7 @@
     <x:xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="50">
     <x:cellStyle name="常规" xfId="0"/>
@@ -1224,7 +1226,7 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="14.399999618530273">
-      <x:c r="A5" s="7">
+      <x:c r="A5" s="8" t="n">
         <x:v>46306.5354914583</x:v>
       </x:c>
       <x:c r="B5" t="s">
@@ -1250,7 +1252,7 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="14.399999618530273">
-      <x:c r="A6" s="7">
+      <x:c r="A6" s="8" t="n">
         <x:v>46306.5354914583</x:v>
       </x:c>
       <x:c r="B6" t="s">
@@ -1276,7 +1278,7 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="7" t="d">
+      <x:c r="A7" s="8" t="d">
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B7" t="str">
@@ -1302,7 +1304,7 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="7" t="d">
+      <x:c r="A8" s="8" t="d">
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B8" t="str">
@@ -1328,7 +1330,7 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="7" t="d">
+      <x:c r="A9" s="8" t="d">
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B9" t="str">
@@ -1354,7 +1356,7 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="7" t="d">
+      <x:c r="A10" s="8" t="d">
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B10" t="str">
@@ -1380,7 +1382,7 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="7" t="d">
+      <x:c r="A11" s="8" t="d">
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B11" t="str">
@@ -1402,7 +1404,7 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="7" t="d">
+      <x:c r="A12" s="8" t="d">
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B12" t="str">
@@ -1424,7 +1426,7 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="7" t="d">
+      <x:c r="A13" s="8" t="d">
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B13" t="str">
@@ -1446,7 +1448,7 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="7" t="d">
+      <x:c r="A14" s="8" t="d">
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B14" t="str">
@@ -1470,7 +1472,7 @@
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="7" t="d">
+      <x:c r="A15" s="8" t="d">
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B15" t="str">
@@ -1492,7 +1494,7 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="7" t="d">
+      <x:c r="A16" s="8" t="d">
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B16" t="str">
@@ -1520,7 +1522,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d5d91d18f5b4d02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbffb03cbefb2405b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Keep only contactable customer leads
</commit_message>
<xml_diff>
--- a/dist/고객관리_연락처기준.xlsx
+++ b/dist/고객관리_연락처기준.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="Rea374cf68841420a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="Rad5c48934c74464b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -38,48 +38,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">근거 링크</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">마스터베어</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">통일상가 B동 2층 2100호</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">남녀 F/W</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">masterbear_golf@naver.com</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">010-3781-6098</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">가을·겨울 OEM·ODM / 바지·재킷</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">https://masterbear580.cafe24.com/</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ELTOO(엘트)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">누죤 1층</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">여성 바지</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">dydxocjswo@naver.com</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">010-5382-0545</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">가을·겨울 OEM·ODM / 여성 팬츠</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">https://www.mininote.co.kr/jobs/?mod=document&amp;uid=140545</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -974,8 +932,8 @@
     <x:tableColumn id="4" name="관심 품목"/>
     <x:tableColumn id="5" name="이메일"/>
     <x:tableColumn id="6" name="휴대폰"/>
-    <x:tableColumn id="12" name="회사주요품목"/>
-    <x:tableColumn id="13" name="근거 링크"/>
+    <x:tableColumn id="7" name="회사주요품목"/>
+    <x:tableColumn id="8" name="근거 링크"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1229,52 +1187,52 @@
       <x:c r="A5" s="8" t="n">
         <x:v>46306.5354914583</x:v>
       </x:c>
-      <x:c r="B5" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="C5" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="D5" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="E5" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="F5" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="G5" s="6" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="H5" t="s">
-        <x:v>16</x:v>
+      <x:c r="B5" t="str">
+        <x:v>마스터베어</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>통일상가 B동 2층 2100호</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>남녀 F/W</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>masterbear_golf@naver.com</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>010-3781-6098</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str">
+        <x:v>가을·겨울 OEM·ODM / 바지·재킷</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>https://masterbear580.cafe24.com/</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="14.399999618530273">
       <x:c r="A6" s="8" t="n">
         <x:v>46306.5354914583</x:v>
       </x:c>
-      <x:c r="B6" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C6" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="D6" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="E6" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="F6" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="G6" s="6" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="H6" t="s">
-        <x:v>23</x:v>
+      <x:c r="B6" t="str">
+        <x:v>ELTOO(엘트)</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>누죤 1층</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>여성 바지</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>dydxocjswo@naver.com</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>010-5382-0545</x:v>
+      </x:c>
+      <x:c r="G6" s="6" t="str">
+        <x:v>가을·겨울 OEM·ODM / 여성 팬츠</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>https://www.mininote.co.kr/jobs/?mod=document&amp;uid=140545</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1386,21 +1344,23 @@
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>뉴골드</x:v>
-      </x:c>
-      <x:c r="C11" t="str">
-        <x:v>통일상가</x:v>
-      </x:c>
+        <x:v>늘봄</x:v>
+      </x:c>
+      <x:c r="C11" t="str"/>
       <x:c r="D11" t="str">
-        <x:v>남성 캐주얼 바지</x:v>
-      </x:c>
-      <x:c r="E11" t="str"/>
-      <x:c r="F11" t="str"/>
+        <x:v>니트·스웨터·가디건, 캐주얼웨어</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>skrmfkd2@naver.com</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>010-6668-6943</x:v>
+      </x:c>
       <x:c r="G11" t="str">
-        <x:v>남성 캐주얼 바지 도매</x:v>
+        <x:v>니트·스웨터·가디건·캐주얼웨어</x:v>
       </x:c>
       <x:c r="H11" t="str">
-        <x:v>공개 채용 공고 확인 · 연락처 확인 필요</x:v>
+        <x:v>사용자 제공 목록</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1408,21 +1368,23 @@
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>하프인치</x:v>
-      </x:c>
-      <x:c r="C12" t="str">
-        <x:v>디오트</x:v>
-      </x:c>
+        <x:v>현지패션</x:v>
+      </x:c>
+      <x:c r="C12" t="str"/>
       <x:c r="D12" t="str">
-        <x:v>여성 바지·원단</x:v>
-      </x:c>
-      <x:c r="E12" t="str"/>
-      <x:c r="F12" t="str"/>
+        <x:v>여성복·남성복·재킷·바지·원피스</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>friends8022@nate.com</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>010-9266-5089</x:v>
+      </x:c>
       <x:c r="G12" t="str">
-        <x:v>여성 팬츠·원단·패턴</x:v>
+        <x:v>여성복·남성복·재킷·바지·원피스</x:v>
       </x:c>
       <x:c r="H12" t="str">
-        <x:v>공개 채용 공고 확인 · 연락처 확인 필요</x:v>
+        <x:v>사용자 제공 목록</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1430,21 +1392,23 @@
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>더베스트오버초이스</x:v>
-      </x:c>
-      <x:c r="C13" t="str">
-        <x:v>통일상가 B동 2층 250·251</x:v>
-      </x:c>
+        <x:v>패턴백화점</x:v>
+      </x:c>
+      <x:c r="C13" t="str"/>
       <x:c r="D13" t="str">
-        <x:v>가을·겨울 바지</x:v>
-      </x:c>
-      <x:c r="E13" t="str"/>
-      <x:c r="F13" t="str"/>
+        <x:v>재킷·코트·점퍼·바지·후드·데님</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>by-song@hanmail.net</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>010-4948-1021</x:v>
+      </x:c>
       <x:c r="G13" t="str">
-        <x:v>가을·겨울 바지·재킷</x:v>
+        <x:v>재킷·코트·점퍼·바지·후드·데님</x:v>
       </x:c>
       <x:c r="H13" t="str">
-        <x:v>고객관리 후보 기록 · 연락처 확인 필요</x:v>
+        <x:v>사용자 제공 목록</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1452,23 +1416,23 @@
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B14" t="str">
-        <x:v>디오트 여성 팬츠 매장 후보</x:v>
-      </x:c>
-      <x:c r="C14" t="str">
-        <x:v>디오트</x:v>
-      </x:c>
+        <x:v>동대문봉제천사</x:v>
+      </x:c>
+      <x:c r="C14" t="str"/>
       <x:c r="D14" t="str">
-        <x:v>여성복·바지</x:v>
-      </x:c>
-      <x:c r="E14" t="str"/>
+        <x:v>셔츠·바지·후드·캐주얼웨어</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>stylook@naver.com</x:v>
+      </x:c>
       <x:c r="F14" t="str">
-        <x:v>02-2117-8000</x:v>
+        <x:v>010-2055-8952</x:v>
       </x:c>
       <x:c r="G14" t="str">
-        <x:v>여성복·잡화 도매 상가</x:v>
+        <x:v>셔츠·바지·후드·캐주얼웨어</x:v>
       </x:c>
       <x:c r="H14" t="str">
-        <x:v>https://dongdaemunmarket.net/board/b03/47537</x:v>
+        <x:v>사용자 제공 목록</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1476,21 +1440,21 @@
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B15" t="str">
-        <x:v>누죤 여성 캐주얼 매장 후보</x:v>
-      </x:c>
-      <x:c r="C15" t="str">
-        <x:v>누죤</x:v>
-      </x:c>
+        <x:v>다올</x:v>
+      </x:c>
+      <x:c r="C15" t="str"/>
       <x:c r="D15" t="str">
-        <x:v>여성 캐주얼·바지</x:v>
+        <x:v>바지·후드·데님·스포츠웨어</x:v>
       </x:c>
       <x:c r="E15" t="str"/>
-      <x:c r="F15" t="str"/>
+      <x:c r="F15" t="str">
+        <x:v>010-3707-2012</x:v>
+      </x:c>
       <x:c r="G15" t="str">
-        <x:v>여성 캐주얼 의류 도매</x:v>
+        <x:v>바지·후드·데님·스포츠웨어</x:v>
       </x:c>
       <x:c r="H15" t="str">
-        <x:v>동대문 도매시장 후보 · 업체별 연락처 확인 필요</x:v>
+        <x:v>사용자 제공 목록 · 공개 이메일 미확인</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1498,21 +1462,21 @@
         <x:v>2026-10-12T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="B16" t="str">
-        <x:v>청평화상가 바지 매장 후보</x:v>
-      </x:c>
-      <x:c r="C16" t="str">
-        <x:v>청평화상가</x:v>
-      </x:c>
+        <x:v>청운어패럴</x:v>
+      </x:c>
+      <x:c r="C16" t="str"/>
       <x:c r="D16" t="str">
-        <x:v>바지·재킷</x:v>
+        <x:v>티셔츠·후드·레깅스·조거팬츠</x:v>
       </x:c>
       <x:c r="E16" t="str"/>
-      <x:c r="F16" t="str"/>
+      <x:c r="F16" t="str">
+        <x:v>010-8840-5646</x:v>
+      </x:c>
       <x:c r="G16" t="str">
-        <x:v>여성 의류·바지 도매</x:v>
+        <x:v>티셔츠·후드·레깅스·조거팬츠</x:v>
       </x:c>
       <x:c r="H16" t="str">
-        <x:v>동대문 도매시장 후보 · 업체별 연락처 확인 필요</x:v>
+        <x:v>사용자 제공 목록 · 공개 이메일 미확인</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1522,7 +1486,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbffb03cbefb2405b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2d3789c8ead41ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Restore Diorot and normalize discovery dates
</commit_message>
<xml_diff>
--- a/dist/고객관리_연락처기준.xlsx
+++ b/dist/고객관리_연락처기준.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="Rad5c48934c74464b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R33d0e089464b4ad4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -924,7 +924,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="발굴일"/>
     <x:tableColumn id="2" name="고객명"/>
@@ -1185,7 +1185,7 @@
     </x:row>
     <x:row r="5" ht="14.399999618530273">
       <x:c r="A5" s="8" t="n">
-        <x:v>46306.5354914583</x:v>
+        <x:v>46306</x:v>
       </x:c>
       <x:c r="B5" t="str">
         <x:v>마스터베어</x:v>
@@ -1211,7 +1211,7 @@
     </x:row>
     <x:row r="6" ht="14.399999618530273">
       <x:c r="A6" s="8" t="n">
-        <x:v>46306.5354914583</x:v>
+        <x:v>46306</x:v>
       </x:c>
       <x:c r="B6" t="str">
         <x:v>ELTOO(엘트)</x:v>
@@ -1236,8 +1236,8 @@
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="8" t="d">
-        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      <x:c r="A7" s="8" t="n">
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="B7" t="str">
         <x:v>남도마켓</x:v>
@@ -1262,8 +1262,8 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="8" t="d">
-        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      <x:c r="A8" s="8" t="n">
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="B8" t="str">
         <x:v>엔디엠(NDM)</x:v>
@@ -1288,8 +1288,8 @@
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="8" t="d">
-        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      <x:c r="A9" s="8" t="n">
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="B9" t="str">
         <x:v>남대문까운사</x:v>
@@ -1314,8 +1314,8 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="8" t="d">
-        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      <x:c r="A10" s="8" t="n">
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="B10" t="str">
         <x:v>URT(로뎀나무아래서)</x:v>
@@ -1340,8 +1340,8 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="8" t="d">
-        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      <x:c r="A11" s="8" t="n">
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="B11" t="str">
         <x:v>늘봄</x:v>
@@ -1364,8 +1364,8 @@
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="8" t="d">
-        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      <x:c r="A12" s="8" t="n">
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="B12" t="str">
         <x:v>현지패션</x:v>
@@ -1388,8 +1388,8 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="8" t="d">
-        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      <x:c r="A13" s="8" t="n">
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="B13" t="str">
         <x:v>패턴백화점</x:v>
@@ -1412,8 +1412,8 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="8" t="d">
-        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      <x:c r="A14" s="8" t="n">
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="B14" t="str">
         <x:v>동대문봉제천사</x:v>
@@ -1436,8 +1436,8 @@
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="8" t="d">
-        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      <x:c r="A15" s="8" t="n">
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="B15" t="str">
         <x:v>다올</x:v>
@@ -1458,8 +1458,8 @@
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="8" t="d">
-        <x:v>2026-10-12T00:00:00.000Z</x:v>
+      <x:c r="A16" s="8" t="n">
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="B16" t="str">
         <x:v>청운어패럴</x:v>
@@ -1477,6 +1477,30 @@
       </x:c>
       <x:c r="H16" t="str">
         <x:v>사용자 제공 목록 · 공개 이메일 미확인</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="8" t="n">
+        <x:v>46307</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>디오트</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>디오트</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>여성복·바지</x:v>
+      </x:c>
+      <x:c r="E17" t="str"/>
+      <x:c r="F17" t="str">
+        <x:v>02-2117-8000</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>여성복·잡화 도매 상가</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>https://dongdaemunmarket.net/board/b03/47537</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1486,7 +1510,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2d3789c8ead41ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b7fc49f447d46d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Seller Ocean contacts
</commit_message>
<xml_diff>
--- a/dist/고객관리_연락처기준.xlsx
+++ b/dist/고객관리_연락처기준.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R33d0e089464b4ad4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="Rc87b7cee72b44fe1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -924,7 +924,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="발굴일"/>
     <x:tableColumn id="2" name="고객명"/>
@@ -1503,6 +1503,61 @@
         <x:v>https://dongdaemunmarket.net/board/b03/47537</x:v>
       </x:c>
     </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="8" t="n">
+        <x:v>46307</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>㈜클로어</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>셀러오션·DDP 쇼룸</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>의류 라이브·동대문 도매 소싱</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>seojw@cloer.co.kr</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>010-8286-2215</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>의류 소싱·라이브커머스·생산 연계</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>https://sellerocean.com/bbs_detail.php?bbs_num=219&amp;g_tb=sns09&amp;id=&amp;pg=&amp;start=&amp;tb=sns09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="8" t="n">
+        <x:v>46307</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>남민우 재고유통·물류</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>셀러오션</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>온라인 브랜드·스마트스토어·쿠팡 셀러 물류</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>oodlesmin@naver.com</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>010-7131-6065</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>브랜드 재고유통·온라인 셀러 물류</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>https://sellerocean.com/bbs_detail.php?b_category=&amp;bbs_num=6292&amp;tb=board_generation_story</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="8"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H1"/>
@@ -1510,7 +1565,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2b7fc49f447d46d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f53e85bff234eb8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add apparel wholesale homepage leads
</commit_message>
<xml_diff>
--- a/dist/고객관리_연락처기준.xlsx
+++ b/dist/고객관리_연락처기준.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="Rc87b7cee72b44fe1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R9c650ea024604724"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -924,7 +924,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="발굴일"/>
     <x:tableColumn id="2" name="고객명"/>
@@ -1556,7 +1556,83 @@
       </x:c>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="8"/>
+      <x:c r="A20" s="8" t="n">
+        <x:v>46308</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>Wstyle</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>온라인 패션 도매</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>패션·의류 B2B 도매</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>help@wstyle.co.kr</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>010-4212-6915</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>사업자 회원 전용 패션·의류 B2B 마켓플레이스</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>https://www.wstyle.co.kr/about</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="8" t="n">
+        <x:v>46308</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>콜라보프로모션</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>동대문·성북구</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>의류 자체제작·도매·프로모션</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>kollabo33@naver.com</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>010-5267-6866</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>의류 프로모션·자체제작·동대문 도매 연계</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>https://www.kollabo.co.kr/default/company/01.php</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="8" t="n">
+        <x:v>46308</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>디디엠애드(DDMAD)</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>동대문</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>여성 의류 도매 B2B</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>ddm_ad@naver.com</x:v>
+      </x:c>
+      <x:c r="F22"/>
+      <x:c r="G22" t="str">
+        <x:v>여성 의류 도매 B2B 쇼핑몰·온라인 컨설팅</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>https://ddmad.co.kr/new/ddmad01.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="8"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1565,7 +1641,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f53e85bff234eb8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14f7b6c8a93547a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add seven apparel and fashion suppliers
</commit_message>
<xml_diff>
--- a/dist/고객관리_연락처기준.xlsx
+++ b/dist/고객관리_연락처기준.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R9c650ea024604724"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="Ra28ba9ee5b70404c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -924,7 +924,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="발굴일"/>
     <x:tableColumn id="2" name="고객명"/>
@@ -1632,7 +1632,183 @@
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="8"/>
+      <x:c r="A23" s="8" t="n">
+        <x:v>46308</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>이유비즈몰</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>온라인 B2B</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>생활·패션 도매</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>mnm10201@naver.com</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>070-4367-3261</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>사업자용 생활·패션 B2B 도매몰</x:v>
+      </x:c>
+      <x:c r="H23" t="str">
+        <x:v>https://www.eyoubizmall.com/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="8" t="n">
+        <x:v>46308</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>정도매</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>온라인 B2B</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>패션의류·잡화 도매</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>jungdome710@gmail.com</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>070-8080-2285</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>사업자 회원 전용 패션의류·잡화 B2B 도매</x:v>
+      </x:c>
+      <x:c r="H24" t="str">
+        <x:v>https://www.jungdome.com/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="8" t="n">
+        <x:v>46308</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>모다허브</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>서울 성동구·의정부</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>의류 전문 3PL·풀필먼트</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>modahub@modahub.co</x:v>
+      </x:c>
+      <x:c r="F25" t="str">
+        <x:v>010-8664-9235</x:v>
+      </x:c>
+      <x:c r="G25" t="str">
+        <x:v>쇼핑몰·브랜드 의류 물류·풀필먼트</x:v>
+      </x:c>
+      <x:c r="H25" t="str">
+        <x:v>https://modahub.co/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="8" t="n">
+        <x:v>46308</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>이음새</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>서울 강북구</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>캐주얼웨어 임가공·생산</x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>wlgjs81@nate.com</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>010-7416-3911</x:v>
+      </x:c>
+      <x:c r="G26" t="str">
+        <x:v>남녀 캐주얼웨어·재킷·바지 임가공</x:v>
+      </x:c>
+      <x:c r="H26" t="str">
+        <x:v>https://www.sfhub.or.kr/page/digital_book_2025.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="8" t="n">
+        <x:v>46308</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>이랑패턴</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>서울 중구</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>정장·캐주얼·기능성웨어 제조</x:v>
+      </x:c>
+      <x:c r="E27"/>
+      <x:c r="F27" t="str">
+        <x:v>02-2256-7702</x:v>
+      </x:c>
+      <x:c r="G27" t="str">
+        <x:v>여성·남성정장·캐주얼·스포츠웨어 패턴·제조</x:v>
+      </x:c>
+      <x:c r="H27" t="str">
+        <x:v>https://sfhub.or.kr/search/04_v?cate=&amp;no=311&amp;page=7&amp;sfl=&amp;size=15&amp;stx=</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="8" t="n">
+        <x:v>46308</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>장안쌤플</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>서울 동대문구</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>캐주얼웨어·스포츠웨어 제조</x:v>
+      </x:c>
+      <x:c r="E28"/>
+      <x:c r="F28" t="str">
+        <x:v>02-2214-8704</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>캐주얼웨어·스포츠·기능성웨어 샘플·제조</x:v>
+      </x:c>
+      <x:c r="H28" t="str">
+        <x:v>https://sfhub.or.kr/search/04_v?cate=&amp;no=318&amp;page=9&amp;sfl=&amp;size=15&amp;stx=</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="8" t="n">
+        <x:v>46308</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>라인로드</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>서울 종로구</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>정장·캐주얼·유니폼 샘플·패턴</x:v>
+      </x:c>
+      <x:c r="E29"/>
+      <x:c r="F29" t="str">
+        <x:v>010-7703-3090</x:v>
+      </x:c>
+      <x:c r="G29" t="str">
+        <x:v>여성·남성정장·캐주얼·유니폼 샘플·패턴</x:v>
+      </x:c>
+      <x:c r="H29" t="str">
+        <x:v>https://sfhub.or.kr/search/04_v?cate=3&amp;no=230&amp;page=0&amp;sfl=&amp;size=&amp;stx=</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="8"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1641,7 +1817,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14f7b6c8a93547a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0238415b06448d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add three verified wholesale suppliers
</commit_message>
<xml_diff>
--- a/dist/고객관리_연락처기준.xlsx
+++ b/dist/고객관리_연락처기준.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="Ra28ba9ee5b70404c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R4cce4f25a0a74d78"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -924,7 +924,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="발굴일"/>
     <x:tableColumn id="2" name="고객명"/>
@@ -1808,7 +1808,85 @@
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="8"/>
+      <x:c r="A30" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>동방섬유</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>동대문종합시장</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>뜨개실·원사·패션 부자재</x:v>
+      </x:c>
+      <x:c r="E30" t="str">
+        <x:v>choish135@gmail.com</x:v>
+      </x:c>
+      <x:c r="F30" t="str">
+        <x:v>010-9074-6268</x:v>
+      </x:c>
+      <x:c r="G30" t="str">
+        <x:v>원사·뜨개실 직접 생산·전국 도매 공급</x:v>
+      </x:c>
+      <x:c r="H30" t="str">
+        <x:v>https://www.dongbangtextile.net/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>고흥수예 본점</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>동대문종합시장 A동</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>커텐·블라인드·이불·베개</x:v>
+      </x:c>
+      <x:c r="E31" t="str">
+        <x:v>ljh920917@naver.com</x:v>
+      </x:c>
+      <x:c r="F31" t="str">
+        <x:v>010-8454-5507</x:v>
+      </x:c>
+      <x:c r="G31" t="str">
+        <x:v>동대문 직영 도매·업소용 맞춤 제작·납품</x:v>
+      </x:c>
+      <x:c r="H31" t="str">
+        <x:v>https://goheungsuye.github.io/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>패션온(FASHION ON)</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>동대문 패션 B2B</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>의류·패션잡화 도소매</x:v>
+      </x:c>
+      <x:c r="E32" t="str">
+        <x:v>ceo@f-on.co.kr</x:v>
+      </x:c>
+      <x:c r="F32" t="str">
+        <x:v>010-4552-6330</x:v>
+      </x:c>
+      <x:c r="G32" t="str">
+        <x:v>동대문 의류·잡화 도소매 거래관리·B2B SCM</x:v>
+      </x:c>
+      <x:c r="H32" t="str">
+        <x:v>https://fashionon.imweb.me/index2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="8"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1817,7 +1895,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0238415b06448d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99fc19c4bbe74683"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Classify wholesale partner by valid email
</commit_message>
<xml_diff>
--- a/dist/고객관리_연락처기준.xlsx
+++ b/dist/고객관리_연락처기준.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R4cce4f25a0a74d78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R249e13dee4f24f41"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -924,7 +924,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="발굴일"/>
     <x:tableColumn id="2" name="고객명"/>
@@ -1886,7 +1886,31 @@
       </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="8"/>
+      <x:c r="A33" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>도매파트너·일진사인</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>온라인 패션 B2B</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>의류 B2B 도매</x:v>
+      </x:c>
+      <x:c r="E33" t="str">
+        <x:v>iljinsign@hanmail.net</x:v>
+      </x:c>
+      <x:c r="F33"/>
+      <x:c r="G33" t="str">
+        <x:v>제조사 직거래 의류 도매 B2B</x:v>
+      </x:c>
+      <x:c r="H33" t="str">
+        <x:v>https://domepartner.co.kr/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="8"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1895,7 +1919,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99fc19c4bbe74683"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e3d98da3cde4ae1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add verified online fashion lead
</commit_message>
<xml_diff>
--- a/dist/고객관리_연락처기준.xlsx
+++ b/dist/고객관리_연락처기준.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R249e13dee4f24f41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="Rfe4ff5b4037d43ec"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -924,7 +924,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="발굴일"/>
     <x:tableColumn id="2" name="고객명"/>
@@ -1910,7 +1910,33 @@
       </x:c>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="8"/>
+      <x:c r="A34" s="8" t="n">
+        <x:v>46310</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>온걸</x:v>
+      </x:c>
+      <x:c r="C34" t="str">
+        <x:v>온라인 패션몰</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>여성 의류·패션잡화</x:v>
+      </x:c>
+      <x:c r="E34" t="str">
+        <x:v>ongirl1000@naver.com</x:v>
+      </x:c>
+      <x:c r="F34" t="str">
+        <x:v>010-5777-7011</x:v>
+      </x:c>
+      <x:c r="G34" t="str">
+        <x:v>온라인 여성 의류 쇼핑몰</x:v>
+      </x:c>
+      <x:c r="H34" t="str">
+        <x:v>https://ongirl.co.kr/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="8"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1919,7 +1945,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e3d98da3cde4ae1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0e6977c2f2a4924"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add ten verified fashion wholesale leads
</commit_message>
<xml_diff>
--- a/dist/고객관리_연락처기준.xlsx
+++ b/dist/고객관리_연락처기준.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="Rfe4ff5b4037d43ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R47d23dbe6ce24a12"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -924,7 +924,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:H44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="발굴일"/>
     <x:tableColumn id="2" name="고객명"/>
@@ -1936,7 +1936,265 @@
       </x:c>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="8"/>
+      <x:c r="A35" s="8" t="n">
+        <x:v>46313</x:v>
+      </x:c>
+      <x:c r="B35" t="str">
+        <x:v>오늘만셀러</x:v>
+      </x:c>
+      <x:c r="C35" t="str">
+        <x:v>온라인 라이브 셀러</x:v>
+      </x:c>
+      <x:c r="D35" t="str">
+        <x:v>동대문 의류·패션·잡화</x:v>
+      </x:c>
+      <x:c r="E35" t="str">
+        <x:v>happy205day@gmail.com</x:v>
+      </x:c>
+      <x:c r="F35" t="str">
+        <x:v>010-7698-9071</x:v>
+      </x:c>
+      <x:c r="G35" t="str">
+        <x:v>패션·뷰티·식품·잡화 라이브 셀러</x:v>
+      </x:c>
+      <x:c r="H35" t="str">
+        <x:v>https://www.onmlive.com/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="8" t="n">
+        <x:v>46313</x:v>
+      </x:c>
+      <x:c r="B36" t="str">
+        <x:v>밤낮커넥트</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
+        <x:v>동대문 B2B</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>의류 도매·사입·3PL</x:v>
+      </x:c>
+      <x:c r="E36" t="str">
+        <x:v>pleatsmom@naver.com</x:v>
+      </x:c>
+      <x:c r="F36" t="str">
+        <x:v>010-5425-9060</x:v>
+      </x:c>
+      <x:c r="G36" t="str">
+        <x:v>동대문 도매업체·라이브셀러 연결 플랫폼</x:v>
+      </x:c>
+      <x:c r="H36" t="str">
+        <x:v>https://bamnatcn.cafe24.com/skin-skin1/seller.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="8" t="n">
+        <x:v>46313</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>BAIE OUD(베이오드)</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>동묘·숭인동</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>여성 의류·우븐·다이마루</x:v>
+      </x:c>
+      <x:c r="E37" t="str">
+        <x:v>xxiyoun246@gmail.com</x:v>
+      </x:c>
+      <x:c r="F37" t="str">
+        <x:v>010-2950-0942</x:v>
+      </x:c>
+      <x:c r="G37" t="str">
+        <x:v>여성 의류 브랜드·생산 핸들링</x:v>
+      </x:c>
+      <x:c r="H37" t="str">
+        <x:v>https://www.mininote.co.kr/jobs/?mod=document&amp;uid=140283</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="8" t="n">
+        <x:v>46313</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>LOUBLLE(루벨르)</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>온라인 패션몰</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>여성 데일리룩·악세서리</x:v>
+      </x:c>
+      <x:c r="E38" t="str">
+        <x:v>hrmc7531@naver.com</x:v>
+      </x:c>
+      <x:c r="F38" t="str">
+        <x:v>010-8717-7215</x:v>
+      </x:c>
+      <x:c r="G38" t="str">
+        <x:v>여성 패션 온라인 쇼핑몰</x:v>
+      </x:c>
+      <x:c r="H38" t="str">
+        <x:v>https://loublle.kr/ko</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="8" t="n">
+        <x:v>46313</x:v>
+      </x:c>
+      <x:c r="B39" t="str">
+        <x:v>미래모자</x:v>
+      </x:c>
+      <x:c r="C39" t="str">
+        <x:v>동대문·평화시장</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
+        <x:v>패션모자·단체모자</x:v>
+      </x:c>
+      <x:c r="E39" t="str">
+        <x:v>mirae2273@daum.net</x:v>
+      </x:c>
+      <x:c r="F39" t="str">
+        <x:v>010-6324-6775</x:v>
+      </x:c>
+      <x:c r="G39" t="str">
+        <x:v>모자 제작·도매 쇼핑몰</x:v>
+      </x:c>
+      <x:c r="H39" t="str">
+        <x:v>https://miraemoja.co.kr/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="8" t="n">
+        <x:v>46313</x:v>
+      </x:c>
+      <x:c r="B40" t="str">
+        <x:v>청림모자</x:v>
+      </x:c>
+      <x:c r="C40" t="str">
+        <x:v>평화시장</x:v>
+      </x:c>
+      <x:c r="D40" t="str">
+        <x:v>캐주얼캡·패션모자</x:v>
+      </x:c>
+      <x:c r="E40" t="str">
+        <x:v>22653575@naver.com</x:v>
+      </x:c>
+      <x:c r="F40" t="str">
+        <x:v>010-8765-9491</x:v>
+      </x:c>
+      <x:c r="G40" t="str">
+        <x:v>모자 도소매·온라인 도매몰</x:v>
+      </x:c>
+      <x:c r="H40" t="str">
+        <x:v>https://www.chunglimmoja.co.kr/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="8" t="n">
+        <x:v>46313</x:v>
+      </x:c>
+      <x:c r="B41" t="str">
+        <x:v>컬러마트</x:v>
+      </x:c>
+      <x:c r="C41" t="str">
+        <x:v>온라인 패션 도매</x:v>
+      </x:c>
+      <x:c r="D41" t="str">
+        <x:v>패션 의류·잡화</x:v>
+      </x:c>
+      <x:c r="E41" t="str">
+        <x:v>hoonbro@naver.com</x:v>
+      </x:c>
+      <x:c r="F41" t="str">
+        <x:v>010-2117-0968</x:v>
+      </x:c>
+      <x:c r="G41" t="str">
+        <x:v>패션 도매 쇼핑몰</x:v>
+      </x:c>
+      <x:c r="H41" t="str">
+        <x:v>https://colormart.kr/product/recent_view_product.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="8" t="n">
+        <x:v>46313</x:v>
+      </x:c>
+      <x:c r="B42" t="str">
+        <x:v>셀러모아</x:v>
+      </x:c>
+      <x:c r="C42" t="str">
+        <x:v>온라인 B2B</x:v>
+      </x:c>
+      <x:c r="D42" t="str">
+        <x:v>패션·잡화·생활용품 도매</x:v>
+      </x:c>
+      <x:c r="E42" t="str">
+        <x:v>support@sellermoa.com</x:v>
+      </x:c>
+      <x:c r="F42"/>
+      <x:c r="G42" t="str">
+        <x:v>도매 상품·마켓 연동 B2B 플랫폼</x:v>
+      </x:c>
+      <x:c r="H42" t="str">
+        <x:v>https://www.sellermoa.com/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="8" t="n">
+        <x:v>46313</x:v>
+      </x:c>
+      <x:c r="B43" t="str">
+        <x:v>글로벌뷰티</x:v>
+      </x:c>
+      <x:c r="C43" t="str">
+        <x:v>온라인 도매몰</x:v>
+      </x:c>
+      <x:c r="D43" t="str">
+        <x:v>미용·패션잡화</x:v>
+      </x:c>
+      <x:c r="E43" t="str">
+        <x:v>gbkyjin@naver.com</x:v>
+      </x:c>
+      <x:c r="F43" t="str">
+        <x:v>010-6793-9876</x:v>
+      </x:c>
+      <x:c r="G43" t="str">
+        <x:v>미용재료·잡화 회원 전용 도매몰</x:v>
+      </x:c>
+      <x:c r="H43" t="str">
+        <x:v>https://globalbeauty.co.kr/index.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="8" t="n">
+        <x:v>46313</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>가로세로 쇼핑몰</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>온라인 종합몰</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>의류·잡화·패션잡화</x:v>
+      </x:c>
+      <x:c r="E44" t="str">
+        <x:v>pandora527@daum.net</x:v>
+      </x:c>
+      <x:c r="F44" t="str">
+        <x:v>010-4775-8253</x:v>
+      </x:c>
+      <x:c r="G44" t="str">
+        <x:v>의류·잡화·패션잡화 종합 쇼핑몰</x:v>
+      </x:c>
+      <x:c r="H44" t="str">
+        <x:v>https://m.grsr.co.kr/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="8"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1945,7 +2203,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0e6977c2f2a4924"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b5d0bc5f6ab4f5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add 10 new customer leads to web app
</commit_message>
<xml_diff>
--- a/dist/고객관리_연락처기준.xlsx
+++ b/dist/고객관리_연락처기준.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R1cb3bb0160d5483b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R38d56b65b9194e2d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2760,33 +2760,7 @@
         <x:v>https://k-jewelry.kr/default/company/company_6.php?sub=04&amp;tit=01</x:v>
       </x:c>
     </x:row>
-    <x:row r="65">
-      <x:c r="A65" s="11" t="d">
-        <x:v>2026-10-20T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="B65" t="str">
-        <x:v>엠셀(Mcell)</x:v>
-      </x:c>
-      <x:c r="C65" t="str">
-        <x:v>경기 성남·안성</x:v>
-      </x:c>
-      <x:c r="D65" t="str">
-        <x:v>스마트웨어·발열 의류 OEM/ODM</x:v>
-      </x:c>
-      <x:c r="E65" t="str">
-        <x:v>contact@mcell.co.kr</x:v>
-      </x:c>
-      <x:c r="F65" t="str">
-        <x:v>070-4333-5233</x:v>
-      </x:c>
-      <x:c r="G65" t="str">
-        <x:v>발열 의류·스마트웨어 소재 개발 및 OEM/ODM</x:v>
-      </x:c>
-      <x:c r="H65" t="str">
-        <x:v>https://www.mcell.co.kr/mcell/oem-odm</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="65" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="65" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A65" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -2799,9 +2773,7 @@
       <x:c r="D65" t="str">
         <x:v>아동복 B2B 도매</x:v>
       </x:c>
-      <x:c r="E65" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="E65" t="str"/>
       <x:c r="F65" t="str">
         <x:v>010-6443-2599</x:v>
       </x:c>
@@ -2812,7 +2784,7 @@
         <x:v>https://www.sellernow.co.kr/post/501961</x:v>
       </x:c>
     </x:row>
-    <x:row r="66" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="66" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A66" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -2825,9 +2797,7 @@
       <x:c r="D66" t="str">
         <x:v>여성의류 B2B 도매</x:v>
       </x:c>
-      <x:c r="E66" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="E66" t="str"/>
       <x:c r="F66" t="str">
         <x:v>010-8780-0823</x:v>
       </x:c>
@@ -2838,7 +2808,7 @@
         <x:v>https://www.sellernow.co.kr/post/500851</x:v>
       </x:c>
     </x:row>
-    <x:row r="67" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="67" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A67" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -2851,9 +2821,7 @@
       <x:c r="D67" t="str">
         <x:v>여성의류 B2B 도매</x:v>
       </x:c>
-      <x:c r="E67" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="E67" t="str"/>
       <x:c r="F67" t="str">
         <x:v>010-4896-9951</x:v>
       </x:c>
@@ -2864,7 +2832,7 @@
         <x:v>https://ozbridge.co.kr/shopinfo/faq.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="68" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="68" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A68" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -2877,9 +2845,7 @@
       <x:c r="D68" t="str">
         <x:v>아동복 B2B 도매</x:v>
       </x:c>
-      <x:c r="E68" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="E68" t="str"/>
       <x:c r="F68" t="str">
         <x:v>010-8113-2213</x:v>
       </x:c>
@@ -2890,7 +2856,7 @@
         <x:v>https://www.sellernow.co.kr/post/501960</x:v>
       </x:c>
     </x:row>
-    <x:row r="69" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="69" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A69" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -2903,9 +2869,7 @@
       <x:c r="D69" t="str">
         <x:v>아동복 자체제작·도매</x:v>
       </x:c>
-      <x:c r="E69" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="E69" t="str"/>
       <x:c r="F69" t="str">
         <x:v>010-6316-8732</x:v>
       </x:c>
@@ -2916,7 +2880,7 @@
         <x:v>https://sellernow.co.kr/post/502008</x:v>
       </x:c>
     </x:row>
-    <x:row r="70" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="70" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A70" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -2942,7 +2906,7 @@
         <x:v>https://www.luardmaison.co.kr/SECRETB2B</x:v>
       </x:c>
     </x:row>
-    <x:row r="71" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="71" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A71" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -2968,7 +2932,7 @@
         <x:v>https://funnydome.com/product/search.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="72" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="72" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A72" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -2994,7 +2958,7 @@
         <x:v>https://maidome.com/goods/populate.php</x:v>
       </x:c>
     </x:row>
-    <x:row r="73" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="73" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A73" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -3020,7 +2984,7 @@
         <x:v>https://www.star-bag.com/store4</x:v>
       </x:c>
     </x:row>
-    <x:row r="74" s="9" customFormat="1" ht="14.4" customHeight="1">
+    <x:row r="74" s="9" customFormat="1" ht="14.399999618530273" customHeight="1">
       <x:c r="A74" s="11" t="n">
         <x:v>46307</x:v>
       </x:c>
@@ -3033,9 +2997,7 @@
       <x:c r="D74" t="str">
         <x:v>의류·패션잡화 B2B 도매</x:v>
       </x:c>
-      <x:c r="E74" t="str">
-        <x:v/>
-      </x:c>
+      <x:c r="E74" t="str"/>
       <x:c r="F74" t="str">
         <x:v>010-7708-2360</x:v>
       </x:c>
@@ -3044,6 +3006,260 @@
       </x:c>
       <x:c r="H74" t="str">
         <x:v>https://www.shinhan.ac.kr/bbs/kr/197/89939/download.do</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>에이팩토리인터내셔널</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>서울 성북구</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>의류 OEM·ODM·원단·부자재</x:v>
+      </x:c>
+      <x:c r="E75" t="str">
+        <x:v>info@a-factory.co.kr</x:v>
+      </x:c>
+      <x:c r="F75" t="str">
+        <x:v>070-4417-6248</x:v>
+      </x:c>
+      <x:c r="G75" t="str">
+        <x:v>국내·중국 의류 생산 및 원부자재 소싱</x:v>
+      </x:c>
+      <x:c r="H75" t="str">
+        <x:v>https://a-factory.co.kr/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>J&amp;G(모노디오)</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>경기 용인</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>스포츠웨어·기능성 원단</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>monodio@naver.com</x:v>
+      </x:c>
+      <x:c r="F76" t="str">
+        <x:v>010-6677-2441</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>국내 의류·원단 OEM/ODM 및 샘플 개발</x:v>
+      </x:c>
+      <x:c r="H76" t="str">
+        <x:v>https://jgapparel.co.kr/ko</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>스와치온</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>서울 성동구</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>패션 원단·부자재</x:v>
+      </x:c>
+      <x:c r="E77" t="str">
+        <x:v>ask@swatchon.com</x:v>
+      </x:c>
+      <x:c r="F77" t="str">
+        <x:v>02-460-4200</x:v>
+      </x:c>
+      <x:c r="G77" t="str">
+        <x:v>동대문 원단 온라인 소싱 플랫폼</x:v>
+      </x:c>
+      <x:c r="H77" t="str">
+        <x:v>https://www.swatchon.com/help/contact</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>브랜딧</x:v>
+      </x:c>
+      <x:c r="C78" t="str">
+        <x:v>경기 양주시</x:v>
+      </x:c>
+      <x:c r="D78" t="str">
+        <x:v>브랜드 포장·택배봉투</x:v>
+      </x:c>
+      <x:c r="E78" t="str">
+        <x:v>with@brand-it.kr</x:v>
+      </x:c>
+      <x:c r="F78"/>
+      <x:c r="G78" t="str">
+        <x:v>온라인 브랜드용 포장재 직접 제조</x:v>
+      </x:c>
+      <x:c r="H78" t="str">
+        <x:v>https://www.brandit.kr/contacts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>골라라</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>서울 동대문</x:v>
+      </x:c>
+      <x:c r="D79" t="str">
+        <x:v>K-패션 도매·수출</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>cs@gollala.me</x:v>
+      </x:c>
+      <x:c r="F79" t="str">
+        <x:v>02-6245-1111</x:v>
+      </x:c>
+      <x:c r="G79" t="str">
+        <x:v>동대문 패션 도매 글로벌 B2B 플랫폼</x:v>
+      </x:c>
+      <x:c r="H79" t="str">
+        <x:v>https://wowseattle.com/wow-posts/hot-deal-forum/294005/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>지비앤케이 인터내셔널</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>서울 마포구</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>의류 OEM·ODM·소싱</x:v>
+      </x:c>
+      <x:c r="E80" t="str">
+        <x:v>contact@gbkay.com</x:v>
+      </x:c>
+      <x:c r="F80" t="str">
+        <x:v>010-9443-4741</x:v>
+      </x:c>
+      <x:c r="G80" t="str">
+        <x:v>의류 생산·무역대행·소싱·물류</x:v>
+      </x:c>
+      <x:c r="H80" t="str">
+        <x:v>https://gbkay.com/production</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>연일섬유</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>서울 종로구·경기 포천</x:v>
+      </x:c>
+      <x:c r="D81" t="str">
+        <x:v>뜨개실·원사·니트 부자재</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>master@yeoniltex.com</x:v>
+      </x:c>
+      <x:c r="F81" t="str">
+        <x:v>02-2263-7117</x:v>
+      </x:c>
+      <x:c r="G81" t="str">
+        <x:v>뜨개실·원사 국내 개발·생산 및 ODM</x:v>
+      </x:c>
+      <x:c r="H81" t="str">
+        <x:v>https://www.yeoniltex.com/odm</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>JMONZ OEM ODM CREW</x:v>
+      </x:c>
+      <x:c r="C82" t="str">
+        <x:v>서울</x:v>
+      </x:c>
+      <x:c r="D82" t="str">
+        <x:v>의류 OEM·ODM·리빙소품</x:v>
+      </x:c>
+      <x:c r="E82" t="str">
+        <x:v>8911a@naver.com</x:v>
+      </x:c>
+      <x:c r="F82" t="str">
+        <x:v>02-555-3975</x:v>
+      </x:c>
+      <x:c r="G82" t="str">
+        <x:v>소량 의류 제작·OEM/ODM·판매 대행</x:v>
+      </x:c>
+      <x:c r="H82" t="str">
+        <x:v>https://jmonz.imweb.me/OEMODM</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B83" t="str">
+        <x:v>드림케이</x:v>
+      </x:c>
+      <x:c r="C83" t="str">
+        <x:v>서울 의류제조</x:v>
+      </x:c>
+      <x:c r="D83" t="str">
+        <x:v>우븐 의류·남녀정장·캐주얼·유니폼</x:v>
+      </x:c>
+      <x:c r="E83"/>
+      <x:c r="F83" t="str">
+        <x:v>010-5201-5649</x:v>
+      </x:c>
+      <x:c r="G83" t="str">
+        <x:v>서울 의류제조 봉제공장 공개 업체</x:v>
+      </x:c>
+      <x:c r="H83" t="str">
+        <x:v>https://www.ksct.or.kr/up_file/202208190303541806873.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="B84" t="str">
+        <x:v>가람패션</x:v>
+      </x:c>
+      <x:c r="C84" t="str">
+        <x:v>서울 의류제조</x:v>
+      </x:c>
+      <x:c r="D84" t="str">
+        <x:v>우븐·토털웨어</x:v>
+      </x:c>
+      <x:c r="E84"/>
+      <x:c r="F84" t="str">
+        <x:v>010-5334-4251</x:v>
+      </x:c>
+      <x:c r="G84" t="str">
+        <x:v>서울 의류제조 봉제공장 공개 업체</x:v>
+      </x:c>
+      <x:c r="H84" t="str">
+        <x:v>https://www.ksct.or.kr/up_file/202208190303541806873.pdf</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3053,7 +3269,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Radc65a55e2e249ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ddc6a6f34664656"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Replace unreachable Dreamcare lead with Sekyung
</commit_message>
<xml_diff>
--- a/dist/고객관리_연락처기준.xlsx
+++ b/dist/고객관리_연락처기준.xlsx
@@ -3219,20 +3219,20 @@
         <x:v>2026-10-24</x:v>
       </x:c>
       <x:c r="B83" t="str">
-        <x:v>드림케어</x:v>
+        <x:v>세경실업</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>서울 의류제조</x:v>
+        <x:v>부산</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>우븐 의류·남녀정장·캐주얼·유니폼</x:v>
+        <x:v>아우터 OEM·ODM·샘플 제작</x:v>
       </x:c>
       <x:c r="E83"/>
       <x:c r="F83" t="str">
-        <x:v>010-5201-5649</x:v>
+        <x:v>010-8523-2048</x:v>
       </x:c>
       <x:c r="G83" t="str">
-        <x:v>서울 의류제조 봉제공장 공개 업체</x:v>
+        <x:v>부산 봉제공장 공개 업체</x:v>
       </x:c>
       <x:c r="H83" t="str">
         <x:v>https://www.ksct.or.kr/up_file/202208190303541806873.pdf</x:v>
@@ -3246,7 +3246,7 @@
         <x:v>가람패션</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>서울 의류제조</x:v>
+        <x:v>부산</x:v>
       </x:c>
       <x:c r="D84" t="str">
         <x:v>우븐·토털웨어</x:v>
@@ -3256,7 +3256,7 @@
         <x:v>010-5334-4251</x:v>
       </x:c>
       <x:c r="G84" t="str">
-        <x:v>서울 의류제조 봉제공장 공개 업체</x:v>
+        <x:v>부산 봉제공장 공개 업체</x:v>
       </x:c>
       <x:c r="H84" t="str">
         <x:v>https://www.ksct.or.kr/up_file/202208190303541806873.pdf</x:v>

</xml_diff>

<commit_message>
Delete Garam Fashion from customer workbook
</commit_message>
<xml_diff>
--- a/dist/고객관리_연락처기준.xlsx
+++ b/dist/고객관리_연락처기준.xlsx
@@ -3238,30 +3238,6 @@
         <x:v>https://www.ksct.or.kr/up_file/202208190303541806873.pdf</x:v>
       </x:c>
     </x:row>
-    <x:row r="84">
-      <x:c r="A84" t="str">
-        <x:v>2026-10-24</x:v>
-      </x:c>
-      <x:c r="B84" t="str">
-        <x:v>가람패션</x:v>
-      </x:c>
-      <x:c r="C84" t="str">
-        <x:v>부산</x:v>
-      </x:c>
-      <x:c r="D84" t="str">
-        <x:v>우븐·토털웨어</x:v>
-      </x:c>
-      <x:c r="E84"/>
-      <x:c r="F84" t="str">
-        <x:v>010-5334-4251</x:v>
-      </x:c>
-      <x:c r="G84" t="str">
-        <x:v>부산 봉제공장 공개 업체</x:v>
-      </x:c>
-      <x:c r="H84" t="str">
-        <x:v>https://www.ksct.or.kr/up_file/202208190303541806873.pdf</x:v>
-      </x:c>
-    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A2:H2"/>

</xml_diff>